<commit_message>
latest updates for 3C break fut
</commit_message>
<xml_diff>
--- a/NIFTY.xlsx
+++ b/NIFTY.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIS\Desktop\Project\3C Break FUT\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88012F6-668C-4810-B099-64F967C49560}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="EQ"/>
+    <sheet name="EQ" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="415">
   <si>
     <t>Sr.no</t>
   </si>
@@ -319,12 +325,6 @@
     <t>NSE:CUMMINSIND-EQ</t>
   </si>
   <si>
-    <t>Cyient Limited</t>
-  </si>
-  <si>
-    <t>NSE:CYIENT-EQ</t>
-  </si>
-  <si>
     <t>DLF Limited</t>
   </si>
   <si>
@@ -457,12 +457,6 @@
     <t>NSE:HDFCLIFE-EQ</t>
   </si>
   <si>
-    <t>HFCL Limited</t>
-  </si>
-  <si>
-    <t>NSE:HFCL-EQ</t>
-  </si>
-  <si>
     <t>Havells India Limited</t>
   </si>
   <si>
@@ -541,12 +535,6 @@
     <t>NSE:IDFCFIRSTB-EQ</t>
   </si>
   <si>
-    <t>IIFL Finance Limited</t>
-  </si>
-  <si>
-    <t>NSE:IIFL-EQ</t>
-  </si>
-  <si>
     <t>ITC Limited</t>
   </si>
   <si>
@@ -571,12 +559,6 @@
     <t>NSE:IOC-EQ</t>
   </si>
   <si>
-    <t>Indian Railway Catering And Tourism Corporation Limited</t>
-  </si>
-  <si>
-    <t>NSE:IRCTC-EQ</t>
-  </si>
-  <si>
     <t>Indian Railway Finance Corporation Limited</t>
   </si>
   <si>
@@ -589,12 +571,6 @@
     <t>NSE:IREDA-EQ</t>
   </si>
   <si>
-    <t>Indraprastha Gas Limited</t>
-  </si>
-  <si>
-    <t>NSE:IGL-EQ</t>
-  </si>
-  <si>
     <t>Indus Towers Limited</t>
   </si>
   <si>
@@ -817,12 +793,6 @@
     <t>NSE:NBCC-EQ</t>
   </si>
   <si>
-    <t>NCC Limited</t>
-  </si>
-  <si>
-    <t>NSE:NCC-EQ</t>
-  </si>
-  <si>
     <t>NHPC Limited</t>
   </si>
   <si>
@@ -1103,12 +1073,6 @@
   </si>
   <si>
     <t>NSE:TATACONSUM-EQ</t>
-  </si>
-  <si>
-    <t>TITAGARH RAIL SYSTEMS LIMITED</t>
-  </si>
-  <si>
-    <t>NSE:TITAGARH-EQ</t>
   </si>
   <si>
     <t>TVS Motor Company Limited</t>
@@ -1306,9 +1270,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1319,6 +1282,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1351,49 +1320,48 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C214" displayName="Table1" name="Table1" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:C214">
-    <filterColumn hiddenButton="1" colId="0"/>
-    <filterColumn hiddenButton="1" colId="1"/>
-    <filterColumn hiddenButton="1" colId="2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:C207" totalsRowShown="0">
+  <autoFilter ref="A1:C207" xr:uid="{00000000-0009-0000-0100-000001000000}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn name="Sr.no" id="1"/>
-    <tableColumn name="Name" id="2"/>
-    <tableColumn name="symbol" id="3"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Sr.no"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="symbol"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="0" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1402,10 +1370,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -1443,71 +1411,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1535,7 +1503,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1558,11 +1526,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1571,13 +1539,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1587,7 +1555,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1596,7 +1564,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1605,7 +1573,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1613,10 +1581,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1681,19 +1649,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C214"/>
+  <dimension ref="A1:C207"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="54.14785714285715" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="34.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.5703125" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1704,7 +1672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row r="2" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1715,7 +1683,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row r="3" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1726,7 +1694,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row r="4" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1737,7 +1705,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row r="5" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1748,7 +1716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row r="6" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1759,7 +1727,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row r="7" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1770,7 +1738,7 @@
         <v>14</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+    <row r="8" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1781,7 +1749,7 @@
         <v>16</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+    <row r="9" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1792,7 +1760,7 @@
         <v>18</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+    <row r="10" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1803,7 +1771,7 @@
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+    <row r="11" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1814,7 +1782,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+    <row r="12" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1825,7 +1793,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+    <row r="13" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1836,7 +1804,7 @@
         <v>26</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+    <row r="14" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1847,7 +1815,7 @@
         <v>28</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+    <row r="15" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -1858,7 +1826,7 @@
         <v>30</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+    <row r="16" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -1869,7 +1837,7 @@
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+    <row r="17" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -1880,7 +1848,7 @@
         <v>34</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+    <row r="18" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1891,7 +1859,7 @@
         <v>36</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+    <row r="19" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1902,7 +1870,7 @@
         <v>38</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+    <row r="20" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1913,7 +1881,7 @@
         <v>40</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+    <row r="21" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1924,7 +1892,7 @@
         <v>42</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+    <row r="22" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1935,7 +1903,7 @@
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+    <row r="23" spans="1:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1946,7 +1914,7 @@
         <v>46</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+    <row r="24" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1957,7 +1925,7 @@
         <v>48</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+    <row r="25" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1968,7 +1936,7 @@
         <v>50</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+    <row r="26" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -1979,7 +1947,7 @@
         <v>52</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+    <row r="27" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -1990,7 +1958,7 @@
         <v>54</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+    <row r="28" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -2001,7 +1969,7 @@
         <v>56</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+    <row r="29" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -2012,7 +1980,7 @@
         <v>58</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+    <row r="30" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2023,7 +1991,7 @@
         <v>60</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
+    <row r="31" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2034,7 +2002,7 @@
         <v>62</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
+    <row r="32" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2045,7 +2013,7 @@
         <v>64</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
+    <row r="33" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2056,7 +2024,7 @@
         <v>66</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
+    <row r="34" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -2067,7 +2035,7 @@
         <v>68</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
+    <row r="35" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -2078,7 +2046,7 @@
         <v>70</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
+    <row r="36" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2089,7 +2057,7 @@
         <v>72</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
+    <row r="37" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -2100,7 +2068,7 @@
         <v>74</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
+    <row r="38" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -2111,7 +2079,7 @@
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
+    <row r="39" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -2122,7 +2090,7 @@
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
+    <row r="40" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2133,7 +2101,7 @@
         <v>80</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
+    <row r="41" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -2144,7 +2112,7 @@
         <v>82</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
+    <row r="42" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -2155,7 +2123,7 @@
         <v>84</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
+    <row r="43" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2166,7 +2134,7 @@
         <v>86</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
+    <row r="44" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2177,7 +2145,7 @@
         <v>88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
+    <row r="45" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -2188,7 +2156,7 @@
         <v>90</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
+    <row r="46" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -2199,7 +2167,7 @@
         <v>92</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
+    <row r="47" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -2210,7 +2178,7 @@
         <v>94</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
+    <row r="48" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -2221,7 +2189,7 @@
         <v>96</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
+    <row r="49" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -2232,7 +2200,7 @@
         <v>98</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
+    <row r="50" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -2243,9 +2211,9 @@
         <v>100</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
+    <row r="51" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>101</v>
@@ -2254,9 +2222,9 @@
         <v>102</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
+    <row r="52" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B52" s="2" t="s">
         <v>103</v>
@@ -2265,9 +2233,9 @@
         <v>104</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
+    <row r="53" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B53" s="2" t="s">
         <v>105</v>
@@ -2276,9 +2244,9 @@
         <v>106</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
+    <row r="54" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B54" s="2" t="s">
         <v>107</v>
@@ -2287,9 +2255,9 @@
         <v>108</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
+    <row r="55" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B55" s="2" t="s">
         <v>109</v>
@@ -2298,9 +2266,9 @@
         <v>110</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
+    <row r="56" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B56" s="2" t="s">
         <v>111</v>
@@ -2309,9 +2277,9 @@
         <v>112</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
+    <row r="57" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B57" s="2" t="s">
         <v>113</v>
@@ -2320,9 +2288,9 @@
         <v>114</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
+    <row r="58" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>115</v>
@@ -2331,9 +2299,9 @@
         <v>116</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
+    <row r="59" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B59" s="2" t="s">
         <v>117</v>
@@ -2342,9 +2310,9 @@
         <v>118</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
+    <row r="60" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B60" s="2" t="s">
         <v>119</v>
@@ -2353,9 +2321,9 @@
         <v>120</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
+    <row r="61" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B61" s="2" t="s">
         <v>121</v>
@@ -2364,9 +2332,9 @@
         <v>122</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
+    <row r="62" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B62" s="2" t="s">
         <v>123</v>
@@ -2375,9 +2343,9 @@
         <v>124</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
+    <row r="63" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B63" s="2" t="s">
         <v>125</v>
@@ -2386,9 +2354,9 @@
         <v>126</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
+    <row r="64" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B64" s="2" t="s">
         <v>127</v>
@@ -2397,9 +2365,9 @@
         <v>128</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
+    <row r="65" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B65" s="2" t="s">
         <v>129</v>
@@ -2408,9 +2376,9 @@
         <v>130</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
+    <row r="66" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B66" s="2" t="s">
         <v>131</v>
@@ -2419,9 +2387,9 @@
         <v>132</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
+    <row r="67" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B67" s="2" t="s">
         <v>133</v>
@@ -2430,9 +2398,9 @@
         <v>134</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
+    <row r="68" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>135</v>
@@ -2441,9 +2409,9 @@
         <v>136</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
+    <row r="69" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B69" s="2" t="s">
         <v>137</v>
@@ -2452,9 +2420,9 @@
         <v>138</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
+    <row r="70" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B70" s="2" t="s">
         <v>139</v>
@@ -2463,9 +2431,9 @@
         <v>140</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
+    <row r="71" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B71" s="2" t="s">
         <v>141</v>
@@ -2474,9 +2442,9 @@
         <v>142</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
+    <row r="72" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B72" s="2" t="s">
         <v>143</v>
@@ -2485,9 +2453,9 @@
         <v>144</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
+    <row r="73" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B73" s="2" t="s">
         <v>145</v>
@@ -2496,9 +2464,9 @@
         <v>146</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
+    <row r="74" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>147</v>
@@ -2507,9 +2475,9 @@
         <v>148</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
+    <row r="75" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>149</v>
@@ -2518,9 +2486,9 @@
         <v>150</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
+    <row r="76" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B76" s="2" t="s">
         <v>151</v>
@@ -2529,9 +2497,9 @@
         <v>152</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
+    <row r="77" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>153</v>
@@ -2540,9 +2508,9 @@
         <v>154</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
+    <row r="78" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>155</v>
@@ -2551,9 +2519,9 @@
         <v>156</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
+    <row r="79" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>157</v>
@@ -2562,9 +2530,9 @@
         <v>158</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
+    <row r="80" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B80" s="2" t="s">
         <v>159</v>
@@ -2573,9 +2541,9 @@
         <v>160</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75">
+    <row r="81" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B81" s="2" t="s">
         <v>161</v>
@@ -2584,9 +2552,9 @@
         <v>162</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75">
+    <row r="82" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>163</v>
@@ -2595,9 +2563,9 @@
         <v>164</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75">
+    <row r="83" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B83" s="2" t="s">
         <v>165</v>
@@ -2606,9 +2574,9 @@
         <v>166</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75">
+    <row r="84" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B84" s="2" t="s">
         <v>167</v>
@@ -2617,9 +2585,9 @@
         <v>168</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75">
+    <row r="85" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>169</v>
@@ -2628,9 +2596,9 @@
         <v>170</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75">
+    <row r="86" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>171</v>
@@ -2639,9 +2607,9 @@
         <v>172</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75">
+    <row r="87" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>173</v>
@@ -2650,9 +2618,9 @@
         <v>174</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75">
+    <row r="88" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>175</v>
@@ -2661,9 +2629,9 @@
         <v>176</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75">
+    <row r="89" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>177</v>
@@ -2672,9 +2640,9 @@
         <v>178</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75">
+    <row r="90" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>179</v>
@@ -2683,9 +2651,9 @@
         <v>180</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75">
+    <row r="91" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>181</v>
@@ -2694,9 +2662,9 @@
         <v>182</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75">
+    <row r="92" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>183</v>
@@ -2705,9 +2673,9 @@
         <v>184</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75">
+    <row r="93" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>185</v>
@@ -2716,9 +2684,9 @@
         <v>186</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75">
+    <row r="94" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>187</v>
@@ -2727,9 +2695,9 @@
         <v>188</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75">
+    <row r="95" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>189</v>
@@ -2738,9 +2706,9 @@
         <v>190</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75">
+    <row r="96" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>191</v>
@@ -2749,9 +2717,9 @@
         <v>192</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75">
+    <row r="97" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>193</v>
@@ -2760,9 +2728,9 @@
         <v>194</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75">
+    <row r="98" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>195</v>
@@ -2771,9 +2739,9 @@
         <v>196</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75">
+    <row r="99" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>197</v>
@@ -2782,9 +2750,9 @@
         <v>198</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75">
+    <row r="100" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>199</v>
@@ -2793,9 +2761,9 @@
         <v>200</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75">
+    <row r="101" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>201</v>
@@ -2804,9 +2772,9 @@
         <v>202</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
+    <row r="102" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>203</v>
@@ -2815,9 +2783,9 @@
         <v>204</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
+    <row r="103" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>205</v>
@@ -2826,9 +2794,9 @@
         <v>206</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
+    <row r="104" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>207</v>
@@ -2837,9 +2805,9 @@
         <v>208</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
+    <row r="105" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>209</v>
@@ -2848,9 +2816,9 @@
         <v>210</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+    <row r="106" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>211</v>
@@ -2859,9 +2827,9 @@
         <v>212</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+    <row r="107" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>213</v>
@@ -2870,9 +2838,9 @@
         <v>214</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+    <row r="108" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>215</v>
@@ -2881,9 +2849,9 @@
         <v>216</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+    <row r="109" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>217</v>
@@ -2892,9 +2860,9 @@
         <v>218</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+    <row r="110" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>219</v>
@@ -2903,9 +2871,9 @@
         <v>220</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+    <row r="111" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>221</v>
@@ -2914,9 +2882,9 @@
         <v>222</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
+    <row r="112" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>223</v>
@@ -2925,9 +2893,9 @@
         <v>224</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
+    <row r="113" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>225</v>
@@ -2936,9 +2904,9 @@
         <v>226</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
+    <row r="114" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>227</v>
@@ -2947,9 +2915,9 @@
         <v>228</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+    <row r="115" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>229</v>
@@ -2958,9 +2926,9 @@
         <v>230</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+    <row r="116" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>231</v>
@@ -2969,9 +2937,9 @@
         <v>232</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+    <row r="117" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>233</v>
@@ -2980,9 +2948,9 @@
         <v>234</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+    <row r="118" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>235</v>
@@ -2991,9 +2959,9 @@
         <v>236</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+    <row r="119" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>237</v>
@@ -3002,9 +2970,9 @@
         <v>238</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+    <row r="120" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B120" s="2" t="s">
         <v>239</v>
@@ -3013,9 +2981,9 @@
         <v>240</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
+    <row r="121" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B121" s="2" t="s">
         <v>241</v>
@@ -3024,9 +2992,9 @@
         <v>242</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
+    <row r="122" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>243</v>
@@ -3035,9 +3003,9 @@
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
+    <row r="123" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B123" s="2" t="s">
         <v>245</v>
@@ -3046,9 +3014,9 @@
         <v>246</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
+    <row r="124" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>247</v>
@@ -3057,9 +3025,9 @@
         <v>248</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
+    <row r="125" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>249</v>
@@ -3068,9 +3036,9 @@
         <v>250</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
+    <row r="126" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>251</v>
@@ -3079,9 +3047,9 @@
         <v>252</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
+    <row r="127" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>253</v>
@@ -3090,9 +3058,9 @@
         <v>254</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
+    <row r="128" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>255</v>
@@ -3101,9 +3069,9 @@
         <v>256</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75">
+    <row r="129" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>257</v>
@@ -3112,9 +3080,9 @@
         <v>258</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75">
+    <row r="130" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>259</v>
@@ -3123,9 +3091,9 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75">
+    <row r="131" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>261</v>
@@ -3134,9 +3102,9 @@
         <v>262</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75">
+    <row r="132" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>263</v>
@@ -3145,9 +3113,9 @@
         <v>264</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75">
+    <row r="133" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>265</v>
@@ -3156,9 +3124,9 @@
         <v>266</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75">
+    <row r="134" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>267</v>
@@ -3167,9 +3135,9 @@
         <v>268</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75">
+    <row r="135" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>269</v>
@@ -3178,9 +3146,9 @@
         <v>270</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75">
+    <row r="136" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>271</v>
@@ -3189,9 +3157,9 @@
         <v>272</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75">
+    <row r="137" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>273</v>
@@ -3200,9 +3168,9 @@
         <v>274</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75">
+    <row r="138" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A138" s="3">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>275</v>
@@ -3211,9 +3179,9 @@
         <v>276</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75">
+    <row r="139" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>277</v>
@@ -3222,9 +3190,9 @@
         <v>278</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75">
+    <row r="140" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A140" s="3">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>279</v>
@@ -3233,9 +3201,9 @@
         <v>280</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75">
+    <row r="141" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A141" s="3">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>281</v>
@@ -3244,9 +3212,9 @@
         <v>282</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75">
+    <row r="142" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A142" s="3">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>283</v>
@@ -3255,9 +3223,9 @@
         <v>284</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75">
+    <row r="143" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A143" s="3">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>285</v>
@@ -3266,9 +3234,9 @@
         <v>286</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75">
+    <row r="144" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A144" s="3">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>287</v>
@@ -3277,9 +3245,9 @@
         <v>288</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75">
+    <row r="145" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A145" s="3">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>289</v>
@@ -3288,9 +3256,9 @@
         <v>290</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75">
+    <row r="146" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A146" s="3">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>291</v>
@@ -3299,9 +3267,9 @@
         <v>292</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75">
+    <row r="147" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A147" s="3">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>293</v>
@@ -3310,9 +3278,9 @@
         <v>294</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75">
+    <row r="148" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="3">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>295</v>
@@ -3321,9 +3289,9 @@
         <v>296</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75">
+    <row r="149" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="3">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>297</v>
@@ -3332,9 +3300,9 @@
         <v>298</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75">
+    <row r="150" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A150" s="3">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>299</v>
@@ -3343,9 +3311,9 @@
         <v>300</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75">
+    <row r="151" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A151" s="3">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>301</v>
@@ -3354,9 +3322,9 @@
         <v>302</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75">
+    <row r="152" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A152" s="3">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>303</v>
@@ -3365,9 +3333,9 @@
         <v>304</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75">
+    <row r="153" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="3">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>305</v>
@@ -3376,9 +3344,9 @@
         <v>306</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75">
+    <row r="154" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A154" s="3">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>307</v>
@@ -3387,9 +3355,9 @@
         <v>308</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75">
+    <row r="155" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="3">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>309</v>
@@ -3398,9 +3366,9 @@
         <v>310</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75">
+    <row r="156" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A156" s="3">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>311</v>
@@ -3409,9 +3377,9 @@
         <v>312</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75">
+    <row r="157" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>313</v>
@@ -3420,9 +3388,9 @@
         <v>314</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75">
+    <row r="158" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>315</v>
@@ -3431,9 +3399,9 @@
         <v>316</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75">
+    <row r="159" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A159" s="3">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>317</v>
@@ -3442,9 +3410,9 @@
         <v>318</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75">
+    <row r="160" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A160" s="3">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>319</v>
@@ -3453,9 +3421,9 @@
         <v>320</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75">
+    <row r="161" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A161" s="3">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>321</v>
@@ -3464,9 +3432,9 @@
         <v>322</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75">
+    <row r="162" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A162" s="3">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>323</v>
@@ -3475,9 +3443,9 @@
         <v>324</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75">
+    <row r="163" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>325</v>
@@ -3486,9 +3454,9 @@
         <v>326</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75">
+    <row r="164" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A164" s="3">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>327</v>
@@ -3497,9 +3465,9 @@
         <v>328</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75">
+    <row r="165" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A165" s="3">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>329</v>
@@ -3508,9 +3476,9 @@
         <v>330</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75">
+    <row r="166" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A166" s="3">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>331</v>
@@ -3519,9 +3487,9 @@
         <v>332</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75">
+    <row r="167" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>333</v>
@@ -3530,9 +3498,9 @@
         <v>334</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75">
+    <row r="168" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="3">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>335</v>
@@ -3541,9 +3509,9 @@
         <v>336</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75">
+    <row r="169" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="3">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>337</v>
@@ -3552,9 +3520,9 @@
         <v>338</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75">
+    <row r="170" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="3">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>339</v>
@@ -3563,9 +3531,9 @@
         <v>340</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
+    <row r="171" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A171" s="3">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>341</v>
@@ -3574,9 +3542,9 @@
         <v>342</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75">
+    <row r="172" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A172" s="3">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>343</v>
@@ -3585,9 +3553,9 @@
         <v>344</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75">
+    <row r="173" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="3">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>345</v>
@@ -3596,9 +3564,9 @@
         <v>346</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75">
+    <row r="174" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A174" s="3">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>347</v>
@@ -3607,9 +3575,9 @@
         <v>348</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75">
+    <row r="175" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A175" s="3">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="B175" s="2" t="s">
         <v>349</v>
@@ -3618,9 +3586,9 @@
         <v>350</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75">
+    <row r="176" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>351</v>
@@ -3629,9 +3597,9 @@
         <v>352</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75">
+    <row r="177" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A177" s="3">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>353</v>
@@ -3640,9 +3608,9 @@
         <v>354</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75">
+    <row r="178" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A178" s="3">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>355</v>
@@ -3651,9 +3619,9 @@
         <v>356</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75">
+    <row r="179" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="3">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>357</v>
@@ -3662,9 +3630,9 @@
         <v>358</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75">
+    <row r="180" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="3">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>359</v>
@@ -3673,9 +3641,9 @@
         <v>360</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75">
+    <row r="181" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A181" s="3">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>361</v>
@@ -3684,9 +3652,9 @@
         <v>362</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75">
+    <row r="182" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A182" s="3">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>363</v>
@@ -3695,9 +3663,9 @@
         <v>364</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75">
+    <row r="183" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A183" s="3">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>365</v>
@@ -3706,9 +3674,9 @@
         <v>366</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
+    <row r="184" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A184" s="3">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B184" s="2" t="s">
         <v>367</v>
@@ -3717,9 +3685,9 @@
         <v>368</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
+    <row r="185" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A185" s="3">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="B185" s="2" t="s">
         <v>369</v>
@@ -3728,9 +3696,9 @@
         <v>370</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
+    <row r="186" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A186" s="3">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>371</v>
@@ -3739,9 +3707,9 @@
         <v>372</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
+    <row r="187" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="3">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B187" s="2" t="s">
         <v>373</v>
@@ -3750,9 +3718,9 @@
         <v>374</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
+    <row r="188" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="3">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>375</v>
@@ -3761,9 +3729,9 @@
         <v>376</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
+    <row r="189" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A189" s="3">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>377</v>
@@ -3772,9 +3740,9 @@
         <v>378</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
+    <row r="190" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A190" s="3">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>379</v>
@@ -3783,9 +3751,9 @@
         <v>380</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
+    <row r="191" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A191" s="3">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>381</v>
@@ -3794,9 +3762,9 @@
         <v>382</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
+    <row r="192" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A192" s="3">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>383</v>
@@ -3805,9 +3773,9 @@
         <v>384</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
+    <row r="193" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A193" s="3">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>385</v>
@@ -3816,9 +3784,9 @@
         <v>386</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
+    <row r="194" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A194" s="3">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>387</v>
@@ -3827,9 +3795,9 @@
         <v>388</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
+    <row r="195" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A195" s="3">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>389</v>
@@ -3838,9 +3806,9 @@
         <v>390</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
+    <row r="196" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A196" s="3">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>391</v>
@@ -3849,9 +3817,9 @@
         <v>392</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
+    <row r="197" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A197" s="3">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>393</v>
@@ -3860,9 +3828,9 @@
         <v>394</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75">
+    <row r="198" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="3">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>395</v>
@@ -3871,9 +3839,9 @@
         <v>396</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75">
+    <row r="199" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A199" s="3">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>397</v>
@@ -3882,9 +3850,9 @@
         <v>398</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75">
+    <row r="200" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A200" s="3">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B200" s="2" t="s">
         <v>399</v>
@@ -3893,9 +3861,9 @@
         <v>400</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75">
+    <row r="201" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A201" s="3">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B201" s="2" t="s">
         <v>401</v>
@@ -3904,9 +3872,9 @@
         <v>402</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75">
+    <row r="202" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A202" s="3">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>403</v>
@@ -3915,9 +3883,9 @@
         <v>404</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75">
+    <row r="203" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B203" s="2" t="s">
         <v>405</v>
@@ -3926,9 +3894,9 @@
         <v>406</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75">
+    <row r="204" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A204" s="3">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>407</v>
@@ -3937,9 +3905,9 @@
         <v>408</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75">
+    <row r="205" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A205" s="3">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B205" s="2" t="s">
         <v>409</v>
@@ -3948,9 +3916,9 @@
         <v>410</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75">
+    <row r="206" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A206" s="3">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>411</v>
@@ -3959,92 +3927,15 @@
         <v>412</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75">
+    <row r="207" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A207" s="3">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>413</v>
       </c>
       <c r="C207" s="2" t="s">
         <v>414</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75">
-      <c r="A208" s="3">
-        <v>207</v>
-      </c>
-      <c r="B208" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="C208" s="2" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75">
-      <c r="A209" s="3">
-        <v>208</v>
-      </c>
-      <c r="B209" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="C209" s="2" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75">
-      <c r="A210" s="3">
-        <v>209</v>
-      </c>
-      <c r="B210" s="2" t="s">
-        <v>419</v>
-      </c>
-      <c r="C210" s="2" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75">
-      <c r="A211" s="3">
-        <v>210</v>
-      </c>
-      <c r="B211" s="2" t="s">
-        <v>421</v>
-      </c>
-      <c r="C211" s="2" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75">
-      <c r="A212" s="3">
-        <v>211</v>
-      </c>
-      <c r="B212" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="C212" s="2" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75">
-      <c r="A213" s="3">
-        <v>212</v>
-      </c>
-      <c r="B213" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="C213" s="2" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75">
-      <c r="A214" s="3">
-        <v>213</v>
-      </c>
-      <c r="B214" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="C214" s="2" t="s">
-        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed nested repo + updated code
</commit_message>
<xml_diff>
--- a/NIFTY.xlsx
+++ b/NIFTY.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIS\Desktop\Project\3C Break FUT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PIS\Desktop\Project\ema9-structure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E88012F6-668C-4810-B099-64F967C49560}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F391FA3-D941-410A-876A-A6B9352A1C70}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="409">
   <si>
     <t>Sr.no</t>
   </si>
@@ -1243,28 +1243,10 @@
     <t>NSE:ZYDUSLIFE-EQ</t>
   </si>
   <si>
-    <t>Sensex</t>
-  </si>
-  <si>
-    <t>BSE:SENSEX-INDEX</t>
-  </si>
-  <si>
-    <t>Gold Petal Futures</t>
-  </si>
-  <si>
-    <t>MCX:GOLDPETAL26JANFUT</t>
-  </si>
-  <si>
-    <t>Sliver Micro Futures</t>
-  </si>
-  <si>
-    <t>MCX:SILVERMIC26FEBFUT</t>
-  </si>
-  <si>
-    <t>Copper Futures</t>
-  </si>
-  <si>
-    <t>MCX:COPPER26JANFUT</t>
+    <t>NIFTY50-INDEX</t>
+  </si>
+  <si>
+    <t>NSE:NIFTY50-INDEX</t>
   </si>
 </sst>
 </file>
@@ -3906,37 +3888,19 @@
       </c>
     </row>
     <row r="205" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A205" s="3">
-        <v>211</v>
-      </c>
-      <c r="B205" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="C205" s="2" t="s">
-        <v>410</v>
-      </c>
+      <c r="A205" s="3"/>
+      <c r="B205" s="2"/>
+      <c r="C205" s="2"/>
     </row>
     <row r="206" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A206" s="3">
-        <v>212</v>
-      </c>
-      <c r="B206" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="C206" s="2" t="s">
-        <v>412</v>
-      </c>
+      <c r="A206" s="3"/>
+      <c r="B206" s="2"/>
+      <c r="C206" s="2"/>
     </row>
     <row r="207" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A207" s="3">
-        <v>213</v>
-      </c>
-      <c r="B207" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="C207" s="2" t="s">
-        <v>414</v>
-      </c>
+      <c r="A207" s="3"/>
+      <c r="B207" s="2"/>
+      <c r="C207" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>